<commit_message>
Add full_distance column to the Scraper sheet in the sample spreadsheet
Keeps the sample file's columns in sync with the real tracking
spreadsheet now that fetch_position.py writes a full_distance value on
the Scraper tab.

Co-Authored-By: Claude Sonnet 5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/helper/sample-files/tracking_sample.xlsx
+++ b/helper/sample-files/tracking_sample.xlsx
@@ -518,7 +518,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:Z3"/>
+  <dimension ref="A1:AA3"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -652,6 +652,11 @@
           <t>cloud_coverage</t>
         </is>
       </c>
+      <c r="AA1" t="inlineStr">
+        <is>
+          <t>full_distance</t>
+        </is>
+      </c>
     </row>
     <row r="2">
       <c r="A2" t="n">
@@ -685,8 +690,6 @@
           <t>Default</t>
         </is>
       </c>
-      <c r="H2" t="inlineStr"/>
-      <c r="I2" t="inlineStr"/>
       <c r="J2" t="inlineStr">
         <is>
           <t>Estonia</t>
@@ -702,15 +705,11 @@
           <t>12 x 4 m</t>
         </is>
       </c>
-      <c r="M2" t="inlineStr"/>
-      <c r="N2" t="inlineStr"/>
-      <c r="O2" t="inlineStr"/>
       <c r="P2" t="inlineStr">
         <is>
           <t>10.4 nm</t>
         </is>
       </c>
-      <c r="Q2" t="inlineStr"/>
       <c r="R2" t="inlineStr">
         <is>
           <t>5.0 Knots</t>
@@ -751,7 +750,9 @@
           <t>62.0 %</t>
         </is>
       </c>
-      <c r="Z2" t="inlineStr"/>
+      <c r="AA2" t="n">
+        <v>500</v>
+      </c>
     </row>
     <row r="3">
       <c r="A3" t="n">
@@ -785,8 +786,6 @@
           <t>Default</t>
         </is>
       </c>
-      <c r="H3" t="inlineStr"/>
-      <c r="I3" t="inlineStr"/>
       <c r="J3" t="inlineStr">
         <is>
           <t>Estonia</t>
@@ -802,15 +801,11 @@
           <t>12 x 4 m</t>
         </is>
       </c>
-      <c r="M3" t="inlineStr"/>
-      <c r="N3" t="inlineStr"/>
-      <c r="O3" t="inlineStr"/>
       <c r="P3" t="inlineStr">
         <is>
           <t>22.1 nm</t>
         </is>
       </c>
-      <c r="Q3" t="inlineStr"/>
       <c r="R3" t="inlineStr">
         <is>
           <t>5.0 Knots</t>
@@ -851,7 +846,9 @@
           <t>65.0 %</t>
         </is>
       </c>
-      <c r="Z3" t="inlineStr"/>
+      <c r="AA3" t="n">
+        <v>511.6511</v>
+      </c>
     </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
@@ -1115,8 +1112,6 @@
           <t>IN Coverage</t>
         </is>
       </c>
-      <c r="E3" t="inlineStr"/>
-      <c r="F3" t="inlineStr"/>
       <c r="G3" t="inlineStr">
         <is>
           <t>4.9 kn</t>

</xml_diff>